<commit_message>
infra-commit fix bulk delete, Resolved React, Implemented proper auth, Excel import funct
</commit_message>
<xml_diff>
--- a/src/templates/import/Laptop.xlsx
+++ b/src/templates/import/Laptop.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\ITAMS\itams-system\src\templates\import\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\app-infra\src\templates\import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B6B4529-9CC1-4608-9959-FF90CFC41C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44AE5780-E794-485A-AD19-EEA5B33CB4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="57">
-  <si>
-    <t>INVENTORY LAPTOP DAIHOA 06/2025</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="56">
   <si>
     <t>Dept</t>
   </si>
@@ -205,17 +202,9 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy/m/d"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -261,49 +250,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -325,40 +277,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -640,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -653,439 +596,424 @@
     <col min="8" max="8" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="23.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:8">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="11"/>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="8" t="s">
+      <c r="B1" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F2" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="8" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="49.5">
+      <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="49.5">
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2">
+        <v>45587</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="16.5">
       <c r="A3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="33">
+      <c r="A4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="16.5">
+      <c r="A5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="33">
+      <c r="A6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2">
-        <v>45587</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="16.5">
-      <c r="A4" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="33">
-      <c r="A5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="3" t="s">
+    </row>
+    <row r="7" spans="1:8" ht="16.5">
+      <c r="A7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="33">
+      <c r="A8" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="30">
+      <c r="A9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="16.5">
+      <c r="A10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="16.5">
-      <c r="A6" s="6" t="s">
+      <c r="B10" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="33">
-      <c r="A7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="16.5">
-      <c r="A8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="33">
-      <c r="A9" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="30">
-      <c r="A10" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="F10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H10" s="7" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="16.5">
       <c r="A11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="F11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H11" s="7" t="s">
         <v>42</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="16.5">
       <c r="A12" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="16.5">
       <c r="A13" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="16.5">
       <c r="A14" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>46</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="16.5">
       <c r="A15" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>47</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="16.5">
       <c r="A16" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>48</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="16.5">
-      <c r="A17" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>50</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
infra-commit fix Excel import funct, Excel export funct
</commit_message>
<xml_diff>
--- a/src/templates/import/Laptop.xlsx
+++ b/src/templates/import/Laptop.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\app-infra\src\templates\import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44AE5780-E794-485A-AD19-EEA5B33CB4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2EFFD55-1FC1-41CD-A1EE-69EFC287B4D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -626,11 +626,11 @@
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>6</v>
       </c>
       <c r="D2" s="2">
         <v>45587</v>
@@ -653,10 +653,10 @@
         <v>8</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>11</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>12</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>13</v>
@@ -678,11 +678,11 @@
       <c r="A4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>18</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>19</v>
@@ -705,10 +705,10 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>24</v>
@@ -730,11 +730,11 @@
       <c r="A6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>29</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>19</v>
@@ -756,11 +756,11 @@
       <c r="A7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>32</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>24</v>
@@ -782,11 +782,11 @@
       <c r="A8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>35</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>36</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>37</v>
@@ -808,11 +808,11 @@
       <c r="A9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>24</v>
@@ -834,11 +834,11 @@
       <c r="A10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>41</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>24</v>
@@ -860,11 +860,11 @@
       <c r="A11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>24</v>
@@ -882,15 +882,15 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="16.5">
+    <row r="12" spans="1:8" ht="30">
       <c r="A12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>44</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>24</v>
@@ -908,15 +908,15 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="16.5">
+    <row r="13" spans="1:8" ht="30">
       <c r="A13" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>24</v>
@@ -938,11 +938,11 @@
       <c r="A14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>46</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>24</v>
@@ -964,11 +964,11 @@
       <c r="A15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>24</v>
@@ -990,11 +990,11 @@
       <c r="A16" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
infra-commit fix error and add auto mapping fiedls in import excel
</commit_message>
<xml_diff>
--- a/src/templates/import/Laptop.xlsx
+++ b/src/templates/import/Laptop.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\app-infra\src\templates\import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2EFFD55-1FC1-41CD-A1EE-69EFC287B4D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F6A5652-281F-41E2-B494-2CDCD94FBB78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -180,12 +180,6 @@
     <t>Barcode</t>
   </si>
   <si>
-    <t>SAP_Barcode</t>
-  </si>
-  <si>
-    <t>Date_buy</t>
-  </si>
-  <si>
     <t>User</t>
   </si>
   <si>
@@ -193,6 +187,12 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t>SAPBarcode</t>
+  </si>
+  <si>
+    <t>DateBuy</t>
   </si>
 </sst>
 </file>
@@ -604,22 +604,22 @@
         <v>50</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>52</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>54</v>
       </c>
       <c r="G1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="49.5">

</xml_diff>